<commit_message>
fix: page4 社区TOP10 + ok/region术语改中文(精确/区级质心)
</commit_message>
<xml_diff>
--- a/DATA/analysis/图数表出图_PPT表格汇总.xlsx
+++ b/DATA/analysis/图数表出图_PPT表格汇总.xlsx
@@ -4689,7 +4689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="11" min="1" max="1"/>
@@ -4710,11 +4710,10 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="20" customHeight="1" s="11">
       <c r="A3" s="32" t="inlineStr">
         <is>
-          <t>表A 4 类问题明细（ok 可落图·社区+村）</t>
+          <t>表A 4 类问题明细（精确可落图·社区+村）</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4730,7 @@
       </c>
       <c r="C4" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
       <c r="D4" s="33" t="inlineStr">
@@ -4763,7 +4762,7 @@
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>50.6</t>
+          <t>50.6%</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
@@ -4795,7 +4794,7 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>36.4</t>
+          <t>36.4%</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
@@ -4805,7 +4804,7 @@
       </c>
       <c r="E6" s="34" t="inlineStr">
         <is>
-          <t>主要为道路破损、桥梁损坏、交通设施故障</t>
+          <t>主要为交通信号灯、人行道、车行道等设施破损</t>
         </is>
       </c>
       <c r="F6" s="34" t="inlineStr">
@@ -4827,7 +4826,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.7%</t>
         </is>
       </c>
       <c r="D7" s="35" t="inlineStr">
@@ -4837,7 +4836,7 @@
       </c>
       <c r="E7" s="34" t="inlineStr">
         <is>
-          <t>主要为消防通道占用、器材缺失</t>
+          <t>主要为消防通道占用、消防器材缺失</t>
         </is>
       </c>
       <c r="F7" s="34" t="inlineStr">
@@ -4859,7 +4858,7 @@
       </c>
       <c r="C8" s="35" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.3%</t>
         </is>
       </c>
       <c r="D8" s="35" t="inlineStr">
@@ -4878,11 +4877,10 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="20" customHeight="1" s="11">
       <c r="A10" s="32" t="inlineStr">
         <is>
-          <t>表B 规模总表（有坐标分级）</t>
+          <t>表B 规模总表（分级：精确/区级质心）</t>
         </is>
       </c>
     </row>
@@ -4894,17 +4892,17 @@
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
-          <t>ok 社区</t>
+          <t>精确社区</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>ok 村</t>
+          <t>精确村</t>
         </is>
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>region 区级</t>
+          <t>区级质心</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
@@ -4914,7 +4912,7 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4944,7 @@
       </c>
       <c r="F12" s="35" t="inlineStr">
         <is>
-          <t>50.6</t>
+          <t>50.6%</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4976,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>36.4</t>
+          <t>36.4%</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5008,7 @@
       </c>
       <c r="F14" s="35" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.7%</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5040,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.3%</t>
         </is>
       </c>
     </row>
@@ -5074,21 +5072,21 @@
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="11">
       <c r="A17" s="37" t="inlineStr">
         <is>
-          <t>口径链：全量 5,005 → 有坐标 2,657（ok 1,713 + region 944）→ ok 可落图 1,529（社区 1,491 + 村 38）</t>
+          <t>口径链：全量 5,005 → 有坐标 2,657（精确 1,713 + 区级质心 944）→ 精确可落图 1,529（社区 1,491 + 村 38）</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" s="11">
       <c r="A18" s="32" t="inlineStr">
         <is>
-          <t>表C 社区 TOP8（ok 点·社区口径）</t>
+          <t>表C 社区 TOP10（精确点·社区口径）</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5108,7 @@
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -5135,7 +5133,7 @@
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="E20" s="34" t="inlineStr">
@@ -5160,12 +5158,12 @@
       </c>
       <c r="D21" s="35" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="E21" s="34" t="inlineStr">
         <is>
-          <t>管网 50、出行安全 30</t>
+          <t>管网 50、出行安全 30、消防 8</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5183,7 @@
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="E22" s="34" t="inlineStr">
@@ -5210,12 +5208,12 @@
       </c>
       <c r="D23" s="35" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="E23" s="34" t="inlineStr">
         <is>
-          <t>管网 26、消防 11</t>
+          <t>管网 26、出行安全 10、消防 11</t>
         </is>
       </c>
     </row>
@@ -5235,12 +5233,12 @@
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
-          <t>2.9</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="E24" s="34" t="inlineStr">
         <is>
-          <t>管网 25</t>
+          <t>管网 25、出行安全 18、消防 2</t>
         </is>
       </c>
     </row>
@@ -5260,12 +5258,12 @@
       </c>
       <c r="D25" s="35" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>出行安全 19</t>
+          <t>管网 17、出行安全 19、消防 5</t>
         </is>
       </c>
     </row>
@@ -5285,12 +5283,12 @@
       </c>
       <c r="D26" s="35" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="E26" s="34" t="inlineStr">
         <is>
-          <t>出行安全 20</t>
+          <t>管网 18、出行安全 20</t>
         </is>
       </c>
     </row>
@@ -5310,136 +5308,156 @@
       </c>
       <c r="D27" s="35" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="E27" s="34" t="inlineStr">
         <is>
-          <t>消防 11</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" s="11">
-      <c r="A29" s="32" t="inlineStr">
-        <is>
-          <t>表D 行政村诉求排行（ok 点·村口径）</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1" s="11">
-      <c r="A30" s="33" t="inlineStr">
+          <t>管网 12、出行安全 15、消防 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" s="11">
+      <c r="A28" s="35" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t>朝阳路社区</t>
+        </is>
+      </c>
+      <c r="C28" s="35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>2.3%</t>
+        </is>
+      </c>
+      <c r="E28" s="34" t="inlineStr">
+        <is>
+          <t>管网 18、出行安全 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="11">
+      <c r="A29" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>香锦社区</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>2.2%</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>管网 20、出行安全 11、消防 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" s="11">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>表D 行政村诉求排行（精确点·村口径）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="11">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>排序</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>村</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C32" s="33" t="inlineStr">
         <is>
           <t>诉求数</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" s="11">
-      <c r="A31" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="34" t="inlineStr">
-        <is>
-          <t>火光村</t>
-        </is>
-      </c>
-      <c r="C31" s="35" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" s="11">
-      <c r="A32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="B32" s="34" t="inlineStr">
-        <is>
-          <t>共升村</t>
-        </is>
-      </c>
-      <c r="C32" s="35" t="inlineStr">
-        <is>
-          <t>10</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1" s="11">
       <c r="A33" s="35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B33" s="34" t="inlineStr">
         <is>
-          <t>灵宝村</t>
+          <t>火光村</t>
         </is>
       </c>
       <c r="C33" s="35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1" s="11">
       <c r="A34" s="35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B34" s="34" t="inlineStr">
         <is>
-          <t>旭光村</t>
+          <t>共升村</t>
         </is>
       </c>
       <c r="C34" s="35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1" s="11">
       <c r="A35" s="35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B35" s="34" t="inlineStr">
         <is>
-          <t>共勤村</t>
+          <t>灵宝村</t>
         </is>
       </c>
       <c r="C35" s="35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" s="11">
       <c r="A36" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>联丰村</t>
+          <t>旭光村</t>
         </is>
       </c>
       <c r="C36" s="35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1" s="11">
       <c r="A37" s="35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>共联村</t>
+          <t>共勤村</t>
         </is>
       </c>
       <c r="C37" s="35" t="inlineStr">
@@ -5450,197 +5468,227 @@
     </row>
     <row r="38" ht="22" customHeight="1" s="11">
       <c r="A38" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>联丰村</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1" s="11">
+      <c r="A39" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>共联村</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" s="11">
+      <c r="A40" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="B38" s="34" t="inlineStr">
+      <c r="B40" s="34" t="inlineStr">
         <is>
           <t>共前村</t>
         </is>
       </c>
-      <c r="C38" s="35" t="inlineStr">
+      <c r="C40" s="35" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1" s="11">
-      <c r="A40" s="32" t="inlineStr">
+    <row r="42" ht="20" customHeight="1" s="11">
+      <c r="A42" s="32" t="inlineStr">
         <is>
           <t>表E 双轨对照（page3 体检结果 ↔ 本页市民反映）</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1" s="11">
-      <c r="A41" s="33" t="inlineStr">
+    <row r="43" ht="22" customHeight="1" s="11">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t>主题</t>
         </is>
       </c>
-      <c r="B41" s="33" t="inlineStr">
+      <c r="B43" s="33" t="inlineStr">
         <is>
           <t>体检发现（page3）</t>
         </is>
       </c>
-      <c r="C41" s="33" t="inlineStr">
+      <c r="C43" s="33" t="inlineStr">
         <is>
           <t>市民反映（本页）</t>
         </is>
       </c>
-      <c r="D41" s="33" t="inlineStr">
+      <c r="D43" s="33" t="inlineStr">
         <is>
           <t>判定</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="26" customHeight="1" s="11">
-      <c r="A42" s="35" t="inlineStr">
-        <is>
-          <t>管网安全</t>
-        </is>
-      </c>
-      <c r="B42" s="34" t="inlineStr">
-        <is>
-          <t>燃气 6 栋 + 管线 186 栋</t>
-        </is>
-      </c>
-      <c r="C42" s="34" t="inlineStr">
-        <is>
-          <t>774 条</t>
-        </is>
-      </c>
-      <c r="D42" s="38" t="n"/>
-      <c r="E42" s="34" t="inlineStr">
-        <is>
-          <t>✓ 双证聚焦</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1" s="11">
-      <c r="A43" s="35" t="inlineStr">
-        <is>
-          <t>消防安全</t>
-        </is>
-      </c>
-      <c r="B43" s="34" t="inlineStr">
-        <is>
-          <t>楼道隐患 240 栋</t>
-        </is>
-      </c>
-      <c r="C43" s="34" t="inlineStr">
-        <is>
-          <t>179 条</t>
-        </is>
-      </c>
-      <c r="D43" s="38" t="n"/>
-      <c r="E43" s="34" t="inlineStr">
-        <is>
-          <t>✓ 双证聚焦</t>
         </is>
       </c>
     </row>
     <row r="44" ht="26" customHeight="1" s="11">
       <c r="A44" s="35" t="inlineStr">
         <is>
-          <t>环境安全</t>
+          <t>管网安全</t>
         </is>
       </c>
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>结构 42 + 围护 454（堡坎）</t>
+          <t>燃气 6 栋 + 管线 186 栋</t>
         </is>
       </c>
       <c r="C44" s="34" t="inlineStr">
         <is>
-          <t>20 条</t>
+          <t>774 条</t>
         </is>
       </c>
       <c r="D44" s="38" t="n"/>
       <c r="E44" s="34" t="inlineStr">
         <is>
-          <t>◐ 体检独证</t>
+          <t>✓ 双证聚焦</t>
         </is>
       </c>
     </row>
     <row r="45" ht="26" customHeight="1" s="11">
       <c r="A45" s="35" t="inlineStr">
         <is>
-          <t>出行安全</t>
+          <t>消防安全</t>
         </is>
       </c>
       <c r="B45" s="34" t="inlineStr">
         <is>
-          <t>（体检无对应）</t>
+          <t>楼道隐患 240 栋</t>
         </is>
       </c>
       <c r="C45" s="34" t="inlineStr">
         <is>
-          <t>556 条</t>
+          <t>179 条</t>
         </is>
       </c>
       <c r="D45" s="38" t="n"/>
       <c r="E45" s="34" t="inlineStr">
         <is>
+          <t>✓ 双证聚焦</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1" s="11">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>环境安全</t>
+        </is>
+      </c>
+      <c r="B46" s="34" t="inlineStr">
+        <is>
+          <t>结构 42 + 围护 454（堡坎）</t>
+        </is>
+      </c>
+      <c r="C46" s="34" t="inlineStr">
+        <is>
+          <t>20 条</t>
+        </is>
+      </c>
+      <c r="D46" s="38" t="n"/>
+      <c r="E46" s="34" t="inlineStr">
+        <is>
+          <t>◐ 体检独证</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1" s="11">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>出行安全</t>
+        </is>
+      </c>
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>（体检无对应）</t>
+        </is>
+      </c>
+      <c r="C47" s="34" t="inlineStr">
+        <is>
+          <t>556 条</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="n"/>
+      <c r="E47" s="34" t="inlineStr">
+        <is>
           <t>◑ 市民独证</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="20" customHeight="1" s="11">
-      <c r="A47" s="32" t="inlineStr">
+    <row r="49" ht="20" customHeight="1" s="11">
+      <c r="A49" s="32" t="inlineStr">
         <is>
           <t>表F 口径详注</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1" s="11">
-      <c r="A48" s="37" t="inlineStr">
-        <is>
-          <t>① 数据源 = 12345_治理清洗版（board 直切）+ checkup 图层（坐标）治理产出（CB-30）</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16" customHeight="1" s="11">
-      <c r="A49" s="37" t="inlineStr">
-        <is>
-          <t>② 三级分级：ok 可落图（社区/村 sjoin）/ region 仅区级 / miss 不落</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1" s="11">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>③ 社区与村分别统计，不混淆</t>
+          <t>① 数据源 = 12345_治理清洗版（board 直切）+ checkup 图层（坐标）治理产出（CB-30）</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1" s="11">
       <c r="A51" s="37" t="inlineStr">
         <is>
-          <t>④ 全量（投诉+求助）5,005 = 有坐标 2,657 + 无坐标（miss）约 2,348</t>
+          <t>② 分级：精确（高德 geocode 精确命中坐标·可落图）/ 区级质心（区级兜底坐标·仅区级统计）/ 无坐标（miss·不落图）</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1" s="11">
       <c r="A52" s="37" t="inlineStr">
         <is>
+          <t>③ 社区与村分别统计，不混淆</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1" s="11">
+      <c r="A53" s="37" t="inlineStr">
+        <is>
+          <t>④ 全量（投诉+求助）5,005 = 有坐标 2,657 + 无坐标约 2,348</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1" s="11">
+      <c r="A54" s="37" t="inlineStr">
+        <is>
           <t>数据源：DATA/analysis/page4_安全韧性_市民反映_分析汇总_2026-08-13.md（v3）· 制作：Codex · 2026-08-13</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A52:I52"/>
     <mergeCell ref="A49:I49"/>
     <mergeCell ref="A51:I51"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A31:I31"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A53:I53"/>
     <mergeCell ref="A50:I50"/>
-    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7978,7 +8026,7 @@
       </c>
       <c r="C4" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
       <c r="D4" s="33" t="inlineStr">
@@ -8173,17 +8221,17 @@
       </c>
       <c r="B12" s="33" t="inlineStr">
         <is>
-          <t>ok 社区</t>
+          <t>精确社区</t>
         </is>
       </c>
       <c r="C12" s="33" t="inlineStr">
         <is>
-          <t>ok 村</t>
+          <t>精确村</t>
         </is>
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>region 区级</t>
+          <t>区级质心</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">
@@ -8193,7 +8241,7 @@
       </c>
       <c r="F12" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
     </row>
@@ -8421,7 +8469,7 @@
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>占 ok%</t>
+          <t>占比</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr">
@@ -8680,6 +8728,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="20" customHeight="1" s="11">
       <c r="A33" s="32" t="inlineStr">
         <is>
@@ -8824,6 +8873,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="20" customHeight="1" s="11">
       <c r="A44" s="32" t="inlineStr">
         <is>
@@ -8968,6 +9018,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="20" customHeight="1" s="11">
       <c r="A52" s="32" t="inlineStr">
         <is>

</xml_diff>